<commit_message>
fix: completely remove all static pre-filled test rows; record Login successful with time taken only when user logs in
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -452,16 +452,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -509,52 +509,6 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Authentication</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Appium Android: Login passed</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Authentication</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Appium Android: Login passed</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>PASSED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: record Login successful test case and ensure Passed Tests sheet opens by default
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -4,11 +4,11 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passed Tests" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passed Tests" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failed Tests" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -415,53 +415,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Test Suite</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Total Tests</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Test Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Time (sec)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Pass Rate %</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Appium Android Tests</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Appium Android: Login successful</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
+        <v>0.04</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Appium Android: Registration successful</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Profile Management</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Appium Android: User toggles light mode theme appearance</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -475,41 +532,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>No.</t>
+          <t>Test Suite</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Total Tests</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Test Name</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Time (sec)</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
+          <t>Pass Rate %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Appium Android Tests</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: real-time Excel reporting for profile updates and all user activities
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,52 @@
         <v>0.06</v>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Profile Management</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Appium Android: User updates profile details successfully</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Profile Management</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Appium Android: User updates profile details successfully</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
@@ -569,10 +615,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Keep moments strictly in moments section and remove moments bar from chats tab
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E192"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4840,6 +4840,29 @@
         <v>0.1</v>
       </c>
       <c r="E192" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Appium Android: User switches to Moments rail tab</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E193" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
@@ -4893,10 +4916,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C2" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Configure user Gmail app password in env and untrack env file
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -481,12 +481,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -504,16 +504,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -527,12 +527,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -550,12 +550,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -573,12 +573,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -619,16 +619,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -665,16 +665,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -688,12 +688,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -826,12 +826,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.04</v>
+        <v>0.3</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -872,16 +872,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -923,11 +923,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -969,11 +969,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User verifies OTP and resets password successfully</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1033,16 +1033,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1079,16 +1079,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1102,16 +1102,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Channels tab</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1125,16 +1125,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Communities tab</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,16 +1148,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens SecureAI</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1171,16 +1171,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Channels tab</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1217,16 +1217,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Communities tab</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1240,16 +1240,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1263,12 +1263,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1309,16 +1309,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.3</v>
+        <v>0.04</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1355,16 +1355,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Security Analysis</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User analyzes URL: undefined (undefined)</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1401,16 +1401,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Appium Android: User verifies OTP and resets password successfully</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.16</v>
+        <v>0.04</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1493,12 +1493,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1516,16 +1516,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1539,12 +1539,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1562,16 +1562,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1590,11 +1590,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Channels tab</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1613,11 +1613,11 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Communities tab</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1636,11 +1636,11 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Appium Android: User opens SecureAI</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1663,7 +1663,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1677,16 +1677,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Channels tab</t>
+          <t>Appium Android: User opens profile settings panel</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1700,16 +1700,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Communities tab</t>
+          <t>Appium Android: User uploads custom profile picture from device</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1728,11 +1728,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User updates profile avatar picture</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1746,12 +1746,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1792,16 +1792,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User views automated test suites panel</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1815,16 +1815,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User views automated test suites panel</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1843,11 +1843,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User opens conversation with Web Master</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1861,16 +1861,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Security Analysis</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Appium Android: User analyzes URL: undefined (undefined)</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1884,12 +1884,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1907,16 +1907,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1930,16 +1930,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User opens conversation with Web Master</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1976,16 +1976,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User toggles light mode theme appearance</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2022,16 +2022,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2045,16 +2045,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2068,16 +2068,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2091,12 +2091,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2119,11 +2119,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2142,11 +2142,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2160,16 +2160,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Appium Android: User opens profile settings panel</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2183,16 +2183,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Appium Android: User uploads custom profile picture from device</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2206,12 +2206,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile avatar picture</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2229,16 +2229,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2252,16 +2252,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2275,16 +2275,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Appium Android: User views automated test suites panel</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2298,16 +2298,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Appium Android: User views automated test suites panel</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2321,16 +2321,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Web Master</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2344,16 +2344,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2367,12 +2367,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2395,11 +2395,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2418,11 +2418,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Web Master</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2441,11 +2441,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2459,16 +2459,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2482,16 +2482,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2505,16 +2505,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2528,16 +2528,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2551,12 +2551,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -2574,16 +2574,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2602,11 +2602,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2625,11 +2625,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2648,11 +2648,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2671,11 +2671,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2694,11 +2694,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2712,16 +2712,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2740,11 +2740,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2763,11 +2763,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2786,11 +2786,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2804,16 +2804,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2827,16 +2827,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2850,16 +2850,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2873,16 +2873,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2901,11 +2901,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2924,11 +2924,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2947,11 +2947,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2988,16 +2988,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3011,16 +3011,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3034,12 +3034,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3080,16 +3080,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User sends end-to-end encrypted message</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User toggles light mode theme appearance</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3126,16 +3126,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3154,11 +3154,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3177,11 +3177,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3195,12 +3195,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3218,16 +3218,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3241,12 +3241,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3264,16 +3264,16 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3287,16 +3287,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3310,16 +3310,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3333,16 +3333,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3356,16 +3356,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3384,11 +3384,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3425,16 +3425,16 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User opens profile settings panel</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3448,16 +3448,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3471,16 +3471,16 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User clears chat history for user_1792685085878_5zl5</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3499,11 +3499,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3522,11 +3522,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3540,16 +3540,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User sends end-to-end encrypted message</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3563,16 +3563,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Appium Android: User sends end-to-end encrypted message</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3586,16 +3586,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3609,16 +3609,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3637,11 +3637,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Mobile</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3655,12 +3655,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3678,12 +3678,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3701,12 +3701,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3724,12 +3724,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3747,12 +3747,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User terminates video call session</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -3770,12 +3770,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -3793,16 +3793,16 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3816,16 +3816,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3839,16 +3839,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User initiates encrypted video call</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3862,16 +3862,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User starts screen sharing</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3890,11 +3890,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -3908,16 +3908,16 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Appium Android: User opens profile settings panel</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -3931,16 +3931,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -3954,16 +3954,16 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Appium Android: User clears chat history for user_1792685085878_5zl5</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -3982,11 +3982,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4005,11 +4005,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4023,16 +4023,16 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Appium Android: User sends end-to-end encrypted message</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4051,11 +4051,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4078,7 +4078,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4097,11 +4097,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4120,11 +4120,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4138,12 +4138,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4161,16 +4161,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4184,16 +4184,16 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4207,16 +4207,16 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4230,16 +4230,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates video call session</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4281,11 +4281,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Mobile</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4299,12 +4299,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -4322,16 +4322,16 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted video call</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4345,16 +4345,16 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Appium Android: User starts screen sharing</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4396,11 +4396,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4414,16 +4414,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4437,16 +4437,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4465,11 +4465,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>0.14</v>
+        <v>0.06</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4483,12 +4483,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4506,16 +4506,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4538,7 +4538,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4575,16 +4575,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.14</v>
+        <v>0.06</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4621,16 +4621,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User initiates encrypted video call</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4644,16 +4644,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User terminates video call session</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4667,16 +4667,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4690,16 +4690,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4713,16 +4713,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -4736,16 +4736,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -4810,11 +4810,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -4851,18 +4851,202 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E193" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E201" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
@@ -4916,10 +5100,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="C2" t="n">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add 24h auto-deletion for moments, manual delete button, and transactional email support
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -670,7 +670,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -693,7 +693,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -734,12 +734,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -762,11 +762,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.04</v>
+        <v>0.3</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -780,16 +780,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -808,7 +808,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -826,16 +826,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -854,11 +854,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.3</v>
+        <v>0.04</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -872,16 +872,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: User verifies OTP and resets password successfully</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -900,11 +900,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -923,11 +923,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -941,16 +941,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -964,16 +964,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Appium Android: User verifies OTP and resets password successfully</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -987,16 +987,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1010,16 +1010,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Channels tab</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1033,16 +1033,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: User switches to Communities tab</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1061,11 +1061,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User opens SecureAI</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1084,11 +1084,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,16 +1148,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Appium Android: User opens SecureAI</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1171,16 +1171,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Channels tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1217,16 +1217,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Communities tab</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1240,16 +1240,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1263,16 +1263,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Security Analysis</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User analyzes URL: undefined (undefined)</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1355,16 +1355,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Security Analysis</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Appium Android: User analyzes URL: undefined (undefined)</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1493,16 +1493,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1539,16 +1539,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1562,16 +1562,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1585,16 +1585,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User opens profile settings panel</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1608,16 +1608,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User uploads custom profile picture from device</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1631,16 +1631,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User updates profile avatar picture</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1654,16 +1654,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1682,11 +1682,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Appium Android: User opens profile settings panel</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1700,12 +1700,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Appium Android: User uploads custom profile picture from device</t>
+          <t>Appium Android: User views automated test suites panel</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1723,16 +1723,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile avatar picture</t>
+          <t>Appium Android: User views automated test suites panel</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1746,16 +1746,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User opens conversation with Web Master</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1769,16 +1769,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1792,16 +1792,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Appium Android: User views automated test suites panel</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1815,16 +1815,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Appium Android: User views automated test suites panel</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1884,16 +1884,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User toggles light mode theme appearance</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1907,16 +1907,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1935,11 +1935,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Web Master</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1976,16 +1976,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1999,12 +1999,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2027,11 +2027,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2045,16 +2045,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2068,16 +2068,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2091,16 +2091,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2119,11 +2119,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2142,11 +2142,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2165,11 +2165,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2188,11 +2188,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2211,11 +2211,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2229,12 +2229,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2252,16 +2252,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2275,16 +2275,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2321,12 +2321,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2344,16 +2344,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2367,16 +2367,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2395,11 +2395,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2413,16 +2413,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2436,16 +2436,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2459,16 +2459,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2505,16 +2505,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2528,12 +2528,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2551,16 +2551,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2579,11 +2579,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2602,11 +2602,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2620,12 +2620,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2652,7 +2652,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2694,11 +2694,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2712,16 +2712,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2740,11 +2740,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2763,11 +2763,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2781,16 +2781,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2809,11 +2809,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2873,16 +2873,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2901,11 +2901,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2924,11 +2924,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2947,11 +2947,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2970,11 +2970,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2988,16 +2988,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User sends end-to-end encrypted message</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3011,16 +3011,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User toggles light mode theme appearance</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3034,16 +3034,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3062,11 +3062,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3080,16 +3080,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Appium Android: User sends end-to-end encrypted message</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3126,16 +3126,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Mobile</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3172,12 +3172,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3287,16 +3287,16 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3310,16 +3310,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3333,16 +3333,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User opens profile settings panel</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3379,16 +3379,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User clears chat history for user_1792685085878_5zl5</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3407,11 +3407,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3425,16 +3425,16 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Appium Android: User opens profile settings panel</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3448,16 +3448,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User sends end-to-end encrypted message</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3471,16 +3471,16 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Appium Android: User clears chat history for user_1792685085878_5zl5</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3540,12 +3540,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Appium Android: User sends end-to-end encrypted message</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3563,16 +3563,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3586,12 +3586,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3609,16 +3609,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3632,16 +3632,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User terminates video call session</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3701,16 +3701,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3729,11 +3729,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3752,11 +3752,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates video call session</t>
+          <t>Appium Android: User initiates encrypted video call</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User starts screen sharing</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -3798,11 +3798,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Mobile</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3816,16 +3816,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3839,16 +3839,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted video call</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3862,16 +3862,16 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Appium Android: User starts screen sharing</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3890,11 +3890,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -3913,11 +3913,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -3940,7 +3940,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -3959,11 +3959,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -3982,11 +3982,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4005,11 +4005,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4028,11 +4028,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4051,11 +4051,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4074,11 +4074,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4101,7 +4101,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4120,11 +4120,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4143,11 +4143,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4166,11 +4166,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4193,7 +4193,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4212,11 +4212,11 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4235,11 +4235,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4304,11 +4304,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4322,16 +4322,16 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4345,16 +4345,16 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4391,16 +4391,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4437,16 +4437,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4506,16 +4506,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4529,16 +4529,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User initiates encrypted video call</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4552,16 +4552,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User terminates video call session</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4575,12 +4575,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4598,12 +4598,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4626,11 +4626,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted video call</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4649,7 +4649,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates video call session</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4667,16 +4667,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4690,16 +4690,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4713,16 +4713,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -4736,16 +4736,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -4759,16 +4759,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -4782,16 +4782,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -4805,16 +4805,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -4851,12 +4851,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -4879,11 +4879,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -4902,11 +4902,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -4971,11 +4971,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D200" t="n">

</xml_diff>

<commit_message>
Fix moments 24h retention, resolve voice/video call audio and ringtone issues, add USB reverse port forwarding launcher and sync web & mobile
</commit_message>
<xml_diff>
--- a/Test Cases/Appium_Test_Report.xlsx
+++ b/Test Cases/Appium_Test_Report.xlsx
@@ -458,12 +458,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -481,16 +481,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -504,16 +504,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Channels tab</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -527,16 +527,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Communities tab</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -550,16 +550,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens SecureAI</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -573,16 +573,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -596,12 +596,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Channels tab</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -619,16 +619,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Communities tab</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -642,16 +642,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -665,12 +665,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -693,7 +693,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -711,16 +711,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -734,12 +734,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -757,16 +757,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.3</v>
+        <v>0.14</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -780,16 +780,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Security Analysis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: User analyzes URL: undefined (undefined)</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -803,12 +803,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -831,11 +831,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -849,16 +849,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -877,11 +877,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Appium Android: User verifies OTP and resets password successfully</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -895,16 +895,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.16</v>
+        <v>0.04</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -941,16 +941,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: Registration successful</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -964,12 +964,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -992,11 +992,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1015,11 +1015,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Channels tab</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1038,11 +1038,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Communities tab</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1061,11 +1061,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Appium Android: User opens SecureAI</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1079,16 +1079,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User opens profile settings panel</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1102,16 +1102,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Channels tab</t>
+          <t>Appium Android: User uploads custom profile picture from device</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1125,16 +1125,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Communities tab</t>
+          <t>Appium Android: User updates profile avatar picture</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1153,11 +1153,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1171,12 +1171,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1194,16 +1194,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User views automated test suites panel</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1217,16 +1217,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User views automated test suites panel</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1240,16 +1240,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Web Master</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1286,12 +1286,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Security Analysis</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Appium Android: User analyzes URL: undefined (undefined)</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1309,16 +1309,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1332,16 +1332,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Web Master</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1355,16 +1355,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User opens conversation with Mobile Agent</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User toggles light mode theme appearance</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1401,12 +1401,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1424,16 +1424,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1447,16 +1447,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Appium Android: Registration successful</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1470,12 +1470,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1493,16 +1493,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1521,11 +1521,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1544,11 +1544,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1567,11 +1567,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1585,16 +1585,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Appium Android: User opens profile settings panel</t>
+          <t>Appium Android: User switches to Link Detector tab</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1608,16 +1608,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Appium Android: User uploads custom profile picture from device</t>
+          <t>Appium Android: User switches to Status tab</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1631,16 +1631,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile avatar picture</t>
+          <t>Appium Android: User switches to Calls tab</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1654,16 +1654,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User switches to Chats tab</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1677,16 +1677,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1700,12 +1700,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Appium Android: User views automated test suites panel</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1723,16 +1723,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Appium Android: User views automated test suites panel</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1746,16 +1746,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Web Master</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1769,16 +1769,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Web Master</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Mobile Agent</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1884,16 +1884,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -1930,16 +1930,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1976,16 +1976,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1999,16 +1999,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2027,11 +2027,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2050,11 +2050,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2073,11 +2073,11 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2096,11 +2096,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Link Detector tab</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status tab</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2142,11 +2142,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2165,11 +2165,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2188,11 +2188,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2229,16 +2229,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2252,16 +2252,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2275,16 +2275,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2413,16 +2413,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Global Chat</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2459,16 +2459,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2482,16 +2482,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User sends end-to-end encrypted message</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2505,16 +2505,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User toggles light mode theme appearance</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2528,16 +2528,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2556,11 +2556,11 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2579,11 +2579,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2597,16 +2597,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2620,12 +2620,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2643,16 +2643,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2666,12 +2666,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2689,16 +2689,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2712,16 +2712,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2735,16 +2735,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2758,16 +2758,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2781,16 +2781,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.14</v>
+        <v>0.06</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2809,11 +2809,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2827,16 +2827,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User opens profile settings panel</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2850,16 +2850,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User updates profile details successfully</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2873,16 +2873,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User clears chat history for user_1792685085878_5zl5</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2901,11 +2901,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Status rail tab</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2924,11 +2924,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.14</v>
+        <v>0.06</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2942,16 +2942,16 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Global Chat</t>
+          <t>Appium Android: User sends end-to-end encrypted message</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2970,11 +2970,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2988,16 +2988,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Appium Android: User sends end-to-end encrypted message</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3011,16 +3011,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles light mode theme appearance</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3034,16 +3034,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User switches to Vault rail tab</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3057,16 +3057,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Mobile</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3080,12 +3080,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3103,12 +3103,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3126,12 +3126,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3149,12 +3149,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User terminates video call session</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -3172,12 +3172,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3195,16 +3195,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3218,16 +3218,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3241,16 +3241,16 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User initiates encrypted video call</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3264,12 +3264,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User starts screen sharing</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Panigrahi</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3333,12 +3333,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Appium Android: User opens profile settings panel</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3356,16 +3356,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Appium Android: User updates profile details successfully</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3379,16 +3379,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Appium Android: User clears chat history for user_1792685085878_5zl5</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Status rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3448,12 +3448,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Appium Android: User sends end-to-end encrypted message</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3476,11 +3476,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3522,11 +3522,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3545,11 +3545,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Vault rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3563,16 +3563,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3586,16 +3586,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3609,16 +3609,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3632,16 +3632,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Appium Android: User accepts incoming call</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3655,16 +3655,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates video call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3678,12 +3678,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3706,11 +3706,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Appium Android: User opens conversation with Sonu Mobile</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3724,16 +3724,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3747,16 +3747,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Profile Management</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted video call</t>
+          <t>Appium Android: User toggles dark mode theme appearance</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3770,16 +3770,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Appium Android: User starts screen sharing</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3816,16 +3816,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3839,16 +3839,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3871,7 +3871,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3885,16 +3885,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -3908,12 +3908,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -3936,11 +3936,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -3959,11 +3959,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -3977,16 +3977,16 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4005,11 +4005,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4023,16 +4023,16 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User initiates encrypted video call</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>0.14</v>
+        <v>0.06</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4046,12 +4046,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User terminates video call session</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -4069,16 +4069,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4092,16 +4092,16 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4115,16 +4115,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4138,16 +4138,16 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4170,7 +4170,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4189,11 +4189,11 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4212,11 +4212,11 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Calls rail tab</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4235,11 +4235,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Profile Management</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Appium Android: User toggles dark mode theme appearance</t>
+          <t>Appium Android: User logs out and returns to the login screen</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4276,16 +4276,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4299,16 +4299,16 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4322,12 +4322,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -4345,12 +4345,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -4368,16 +4368,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4391,12 +4391,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4414,12 +4414,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4437,16 +4437,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4460,16 +4460,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4483,12 +4483,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Moments Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Appium Android: User views contact Moment story</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4506,16 +4506,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4529,16 +4529,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted video call</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4552,12 +4552,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates video call session</t>
+          <t>Appium Android: OTP generated and sent to Gmail</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -4575,16 +4575,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4598,16 +4598,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Appium Android: User initiates encrypted voice call</t>
+          <t>Appium Android: Password successfully reset via Gmail OTP</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4621,16 +4621,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Appium Android: User terminates voice call session</t>
+          <t>Appium Android: User verifies OTP and resets password successfully</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4644,12 +4644,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Appium Android: User hangs up call session</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -4667,16 +4667,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Moments rail tab</t>
+          <t>Appium Android: Login successful</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4695,11 +4695,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User switches to Moments rail tab</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4713,16 +4713,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Calls rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -4736,16 +4736,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Appium Android: User switches to Chats rail tab</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>0.14</v>
+        <v>0.04</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -4759,12 +4759,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Appium Android: User logs out and returns to the login screen</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -4782,12 +4782,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Moments Management</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User views contact Moment story</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -4805,16 +4805,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: User switches to Chats rail tab</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -4828,12 +4828,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User opens conversation with Sonu Mobile</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -4851,16 +4851,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -4874,16 +4874,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Appium Android: User requests OTP sent to Gmail for password reset</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -4897,12 +4897,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -4920,16 +4920,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User initiates encrypted voice call</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -4943,12 +4943,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -4966,12 +4966,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -4989,12 +4989,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Appium Android: Password successfully reset via Gmail OTP</t>
+          <t>Appium Android: User accepts incoming call</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5012,12 +5012,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Appium Android: Login successful</t>
+          <t>Appium Android: User terminates voice call session</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Appium Android: OTP generated and sent to Gmail</t>
+          <t>Appium Android: User hangs up call session</t>
         </is>
       </c>
       <c r="D201" t="n">

</xml_diff>